<commit_message>
Control de cambios inspeccion preoperacional
</commit_message>
<xml_diff>
--- a/EquiposUnidos/app/src/main/res/raw/template_inspec_cargador.xlsx
+++ b/EquiposUnidos/app/src/main/res/raw/template_inspec_cargador.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Developer user\android\williApp\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elksi\Android\williApp\EquiposUnidos\app\src\main\res\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A93B6F-75F5-4183-98FB-397FB4B50779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5308662-91CA-4CC4-A65B-78F18C166353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FT-MANT-01" sheetId="4" r:id="rId1"/>
@@ -21,7 +21,6 @@
   </externalReferences>
   <definedNames>
     <definedName name="AÑO">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'FT-MANT-01'!$A$1:$P$34</definedName>
     <definedName name="Cargos">[1]Datos!$D$2:$D$39</definedName>
     <definedName name="CERT">#REF!</definedName>
     <definedName name="CREDITO">#REF!</definedName>
@@ -41,14 +40,28 @@
     <definedName name="MENSAJEERROR2">[2]Hoja1!$D$1</definedName>
     <definedName name="MES">#REF!</definedName>
     <definedName name="PLAZO">#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'FT-MANT-01'!$A$1:$P$38</definedName>
     <definedName name="TIPODEE">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="69">
   <si>
     <t>Señale su respuesta con una ´´X´´</t>
   </si>
@@ -251,7 +264,10 @@
     <t xml:space="preserve">OBSERVACIONES  </t>
   </si>
   <si>
-    <t>fkds</t>
+    <t>CEDULA</t>
+  </si>
+  <si>
+    <t>FIRMA</t>
   </si>
 </sst>
 </file>
@@ -573,7 +589,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="62">
+  <borders count="65">
     <border>
       <left/>
       <right/>
@@ -809,17 +825,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -844,17 +849,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -1306,6 +1300,59 @@
       <right/>
       <top/>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1375,7 +1422,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1393,42 +1440,42 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="26" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="3"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="3"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="3"/>
       <protection hidden="1"/>
     </xf>
@@ -1454,7 +1501,16 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1481,15 +1537,15 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1497,11 +1553,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1513,11 +1569,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1529,11 +1585,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="26" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1552,46 +1608,46 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1606,7 +1662,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1615,7 +1671,7 @@
     <xf numFmtId="0" fontId="25" fillId="26" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="26" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1624,7 +1680,7 @@
     <xf numFmtId="0" fontId="25" fillId="26" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1633,24 +1689,15 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1660,65 +1707,134 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="62">
@@ -1814,7 +1930,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1528286</xdr:colOff>
+      <xdr:colOff>1368266</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>263287</xdr:rowOff>
     </xdr:to>
@@ -2771,109 +2887,109 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <dimension ref="A1:Q50"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" style="1" customWidth="1"/>
-    <col min="4" max="5" width="4.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="4.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" style="1" customWidth="1"/>
     <col min="9" max="9" width="30" style="1" customWidth="1"/>
-    <col min="10" max="11" width="4.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="7.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="37.5703125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="4.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="7.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="37.5546875" style="1" customWidth="1"/>
     <col min="14" max="16" width="8" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="1"/>
+    <col min="17" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21" customHeight="1">
-      <c r="A1" s="38"/>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="42" t="s">
+      <c r="A1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="43"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="46"/>
       <c r="M1" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="46" t="s">
+      <c r="N1" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="46"/>
-      <c r="P1" s="47"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="50"/>
     </row>
     <row r="2" spans="1:16" ht="21" customHeight="1">
-      <c r="A2" s="40"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="45"/>
+      <c r="A2" s="43"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="48"/>
       <c r="M2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="48">
+      <c r="N2" s="51">
         <v>14</v>
       </c>
-      <c r="O2" s="48"/>
-      <c r="P2" s="49"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="52"/>
     </row>
     <row r="3" spans="1:16" ht="21" customHeight="1">
-      <c r="A3" s="40"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="45"/>
+      <c r="A3" s="43"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="48"/>
       <c r="M3" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="50">
+      <c r="N3" s="53">
         <v>45218</v>
       </c>
-      <c r="O3" s="50"/>
-      <c r="P3" s="51"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="54"/>
     </row>
     <row r="4" spans="1:16" ht="6.75" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="53"/>
+      <c r="A4" s="55"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="56"/>
       <c r="N4" s="21"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="55"/>
+      <c r="O4" s="57"/>
+      <c r="P4" s="58"/>
     </row>
     <row r="5" spans="1:16" ht="20.25" customHeight="1">
       <c r="A5" s="2"/>
@@ -2881,23 +2997,23 @@
       <c r="C5" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="57" t="s">
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="J5" s="58"/>
-      <c r="K5" s="58"/>
-      <c r="L5" s="59"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="62"/>
       <c r="M5" s="28" t="s">
         <v>4</v>
       </c>
       <c r="N5" s="23"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="55"/>
+      <c r="O5" s="57"/>
+      <c r="P5" s="58"/>
     </row>
     <row r="6" spans="1:16" ht="20.25" customHeight="1">
       <c r="A6" s="2"/>
@@ -2905,21 +3021,21 @@
       <c r="C6" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="60" t="s">
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="61"/>
-      <c r="K6" s="61"/>
-      <c r="L6" s="62"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
+      <c r="L6" s="65"/>
       <c r="M6" s="28"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="54"/>
-      <c r="P6" s="55"/>
+      <c r="O6" s="57"/>
+      <c r="P6" s="58"/>
     </row>
     <row r="7" spans="1:16" ht="20.25" customHeight="1">
       <c r="A7" s="2"/>
@@ -2927,21 +3043,21 @@
       <c r="C7" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="56"/>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="63" t="s">
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="59"/>
+      <c r="I7" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="J7" s="64"/>
-      <c r="K7" s="64"/>
-      <c r="L7" s="65"/>
+      <c r="J7" s="67"/>
+      <c r="K7" s="67"/>
+      <c r="L7" s="68"/>
       <c r="M7" s="28"/>
       <c r="N7" s="3"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="55"/>
+      <c r="O7" s="57"/>
+      <c r="P7" s="58"/>
     </row>
     <row r="8" spans="1:16" ht="20.25" customHeight="1">
       <c r="A8" s="2"/>
@@ -2949,21 +3065,21 @@
       <c r="C8" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="66" t="s">
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="67"/>
-      <c r="K8" s="67"/>
-      <c r="L8" s="68"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="71"/>
       <c r="M8" s="28"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="54"/>
-      <c r="P8" s="55"/>
+      <c r="O8" s="57"/>
+      <c r="P8" s="58"/>
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="2"/>
@@ -2980,55 +3096,55 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
-      <c r="O9" s="54"/>
-      <c r="P9" s="55"/>
+      <c r="O9" s="57"/>
+      <c r="P9" s="58"/>
     </row>
     <row r="10" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="36"/>
-      <c r="P10" s="37"/>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="39"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
+      <c r="L10" s="39"/>
+      <c r="M10" s="39"/>
+      <c r="N10" s="39"/>
+      <c r="O10" s="39"/>
+      <c r="P10" s="40"/>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="72" t="s">
+      <c r="A11" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="73"/>
-      <c r="J11" s="73"/>
-      <c r="K11" s="73"/>
-      <c r="L11" s="73"/>
-      <c r="M11" s="73"/>
-      <c r="N11" s="73"/>
-      <c r="O11" s="73"/>
-      <c r="P11" s="74"/>
+      <c r="B11" s="76"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
+      <c r="I11" s="76"/>
+      <c r="J11" s="76"/>
+      <c r="K11" s="76"/>
+      <c r="L11" s="76"/>
+      <c r="M11" s="76"/>
+      <c r="N11" s="76"/>
+      <c r="O11" s="76"/>
+      <c r="P11" s="77"/>
     </row>
     <row r="12" spans="1:16" s="16" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A12" s="75" t="s">
+      <c r="A12" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="C12" s="77"/>
+      <c r="B12" s="79"/>
+      <c r="C12" s="80"/>
       <c r="D12" s="11" t="s">
         <v>2</v>
       </c>
@@ -3038,11 +3154,11 @@
       <c r="F12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="78" t="s">
+      <c r="G12" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="H12" s="79"/>
-      <c r="I12" s="80"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="83"/>
       <c r="J12" s="14" t="s">
         <v>2</v>
       </c>
@@ -3066,28 +3182,28 @@
       </c>
     </row>
     <row r="13" spans="1:16" ht="15" customHeight="1">
-      <c r="A13" s="81" t="s">
+      <c r="A13" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="82"/>
-      <c r="C13" s="82"/>
-      <c r="D13" s="111"/>
-      <c r="E13" s="111"/>
-      <c r="F13" s="111"/>
-      <c r="G13" s="83" t="s">
+      <c r="B13" s="85"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="H13" s="83"/>
-      <c r="I13" s="83"/>
-      <c r="J13" s="111"/>
-      <c r="K13" s="111"/>
-      <c r="L13" s="111"/>
+      <c r="H13" s="86"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="30"/>
       <c r="M13" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="N13" s="111"/>
-      <c r="O13" s="111"/>
-      <c r="P13" s="112"/>
+      <c r="N13" s="30"/>
+      <c r="O13" s="30"/>
+      <c r="P13" s="31"/>
     </row>
     <row r="14" spans="1:16" ht="15" customHeight="1">
       <c r="A14" s="6" t="s">
@@ -3095,534 +3211,548 @@
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="26"/>
-      <c r="D14" s="111"/>
-      <c r="E14" s="111"/>
-      <c r="F14" s="111"/>
-      <c r="G14" s="32" t="s">
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="H14" s="33"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="111"/>
-      <c r="K14" s="111"/>
-      <c r="L14" s="111"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
       <c r="M14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="N14" s="111"/>
-      <c r="O14" s="111"/>
-      <c r="P14" s="112"/>
+      <c r="N14" s="30"/>
+      <c r="O14" s="30"/>
+      <c r="P14" s="31"/>
     </row>
     <row r="15" spans="1:16" ht="15" customHeight="1">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="111"/>
-      <c r="E15" s="111"/>
-      <c r="F15" s="111"/>
-      <c r="G15" s="32" t="s">
+      <c r="B15" s="33"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="H15" s="33"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="111"/>
-      <c r="K15" s="111"/>
-      <c r="L15" s="111"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
       <c r="M15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="N15" s="111"/>
-      <c r="O15" s="111"/>
-      <c r="P15" s="112"/>
+      <c r="N15" s="30"/>
+      <c r="O15" s="30"/>
+      <c r="P15" s="31"/>
     </row>
     <row r="16" spans="1:16" ht="15" customHeight="1">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="111" t="s">
-        <v>67</v>
-      </c>
-      <c r="G16" s="32" t="s">
+      <c r="B16" s="33"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="H16" s="33"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="111"/>
-      <c r="K16" s="111"/>
-      <c r="L16" s="111"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
       <c r="M16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="N16" s="111"/>
-      <c r="O16" s="111"/>
-      <c r="P16" s="112"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="30"/>
+      <c r="P16" s="31"/>
     </row>
     <row r="17" spans="1:17" ht="15" customHeight="1">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="111"/>
-      <c r="E17" s="111"/>
-      <c r="F17" s="111"/>
-      <c r="G17" s="32" t="s">
+      <c r="B17" s="33"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="H17" s="33"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="111"/>
-      <c r="K17" s="111"/>
-      <c r="L17" s="111"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
       <c r="M17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="N17" s="111"/>
-      <c r="O17" s="111"/>
-      <c r="P17" s="112"/>
+      <c r="N17" s="30"/>
+      <c r="O17" s="30"/>
+      <c r="P17" s="31"/>
       <c r="Q17" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="15" customHeight="1">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="111"/>
-      <c r="E18" s="111"/>
-      <c r="F18" s="111"/>
-      <c r="G18" s="32" t="s">
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="H18" s="33"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="111"/>
-      <c r="K18" s="111"/>
-      <c r="L18" s="111"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
       <c r="M18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N18" s="111"/>
-      <c r="O18" s="111"/>
-      <c r="P18" s="112"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="30"/>
+      <c r="P18" s="31"/>
     </row>
     <row r="19" spans="1:17" ht="15" customHeight="1">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="111"/>
-      <c r="E19" s="111"/>
-      <c r="F19" s="111"/>
-      <c r="G19" s="32" t="s">
+      <c r="B19" s="33"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="H19" s="33"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="111"/>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="37"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
       <c r="M19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="N19" s="111"/>
-      <c r="O19" s="111"/>
-      <c r="P19" s="112"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="31"/>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="111"/>
-      <c r="E20" s="111"/>
-      <c r="F20" s="111"/>
-      <c r="G20" s="32" t="s">
+      <c r="B20" s="33"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="33"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="111"/>
-      <c r="K20" s="111"/>
-      <c r="L20" s="111"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
       <c r="M20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="N20" s="111"/>
-      <c r="O20" s="111"/>
-      <c r="P20" s="112"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="31"/>
     </row>
     <row r="21" spans="1:17" s="3" customFormat="1" ht="15" customHeight="1">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="111"/>
-      <c r="E21" s="111"/>
-      <c r="F21" s="111"/>
-      <c r="G21" s="32" t="s">
+      <c r="B21" s="33"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="H21" s="33"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="111"/>
-      <c r="K21" s="111"/>
-      <c r="L21" s="111"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30"/>
+      <c r="L21" s="30"/>
       <c r="M21" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N21" s="111"/>
-      <c r="O21" s="111"/>
-      <c r="P21" s="112"/>
+      <c r="N21" s="30"/>
+      <c r="O21" s="30"/>
+      <c r="P21" s="31"/>
     </row>
     <row r="22" spans="1:17" ht="15" customHeight="1">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="111"/>
-      <c r="E22" s="111"/>
-      <c r="F22" s="111"/>
-      <c r="G22" s="32" t="s">
+      <c r="B22" s="33"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="111"/>
-      <c r="K22" s="111"/>
-      <c r="L22" s="111"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
       <c r="M22" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="N22" s="111"/>
-      <c r="O22" s="111"/>
-      <c r="P22" s="112"/>
+      <c r="N22" s="30"/>
+      <c r="O22" s="30"/>
+      <c r="P22" s="31"/>
     </row>
     <row r="23" spans="1:17" ht="15" customHeight="1">
-      <c r="A23" s="29" t="s">
+      <c r="A23" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="111"/>
-      <c r="E23" s="111"/>
-      <c r="F23" s="111"/>
-      <c r="G23" s="32" t="s">
+      <c r="B23" s="33"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="H23" s="33"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="111"/>
-      <c r="K23" s="111"/>
-      <c r="L23" s="111"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="30"/>
+      <c r="L23" s="30"/>
       <c r="M23" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="N23" s="111"/>
-      <c r="O23" s="111"/>
-      <c r="P23" s="112"/>
+      <c r="N23" s="30"/>
+      <c r="O23" s="30"/>
+      <c r="P23" s="31"/>
     </row>
     <row r="24" spans="1:17" ht="15" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="111"/>
-      <c r="E24" s="111"/>
-      <c r="F24" s="111"/>
-      <c r="G24" s="32" t="s">
+      <c r="B24" s="33"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="H24" s="33"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="111"/>
-      <c r="K24" s="111"/>
-      <c r="L24" s="111"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
       <c r="M24" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="N24" s="111"/>
-      <c r="O24" s="111"/>
-      <c r="P24" s="112"/>
+      <c r="N24" s="30"/>
+      <c r="O24" s="30"/>
+      <c r="P24" s="31"/>
     </row>
     <row r="25" spans="1:17" ht="15" customHeight="1">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="111"/>
-      <c r="E25" s="111"/>
-      <c r="F25" s="110"/>
-      <c r="G25" s="32" t="s">
+      <c r="B25" s="33"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="H25" s="33"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="111"/>
-      <c r="K25" s="111"/>
-      <c r="L25" s="111"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="30"/>
+      <c r="K25" s="30"/>
+      <c r="L25" s="30"/>
       <c r="M25" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="N25" s="111"/>
-      <c r="O25" s="111"/>
-      <c r="P25" s="112"/>
+      <c r="N25" s="30"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="31"/>
     </row>
     <row r="26" spans="1:17" ht="15" customHeight="1">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="111"/>
-      <c r="E26" s="111"/>
-      <c r="F26" s="110"/>
-      <c r="G26" s="32" t="s">
+      <c r="B26" s="33"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="H26" s="33"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="111"/>
-      <c r="K26" s="111"/>
-      <c r="L26" s="111"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
       <c r="M26" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="N26" s="111"/>
-      <c r="O26" s="111"/>
-      <c r="P26" s="112"/>
+      <c r="N26" s="30"/>
+      <c r="O26" s="30"/>
+      <c r="P26" s="31"/>
     </row>
     <row r="27" spans="1:17" ht="15" customHeight="1" thickBot="1">
-      <c r="A27" s="84" t="s">
+      <c r="A27" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="85"/>
-      <c r="C27" s="85"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="85"/>
-      <c r="F27" s="85"/>
-      <c r="G27" s="85"/>
-      <c r="H27" s="85"/>
-      <c r="I27" s="85"/>
-      <c r="J27" s="85"/>
-      <c r="K27" s="85"/>
-      <c r="L27" s="85"/>
-      <c r="M27" s="85"/>
-      <c r="N27" s="85"/>
-      <c r="O27" s="85"/>
-      <c r="P27" s="86"/>
+      <c r="B27" s="88"/>
+      <c r="C27" s="88"/>
+      <c r="D27" s="88"/>
+      <c r="E27" s="88"/>
+      <c r="F27" s="88"/>
+      <c r="G27" s="88"/>
+      <c r="H27" s="88"/>
+      <c r="I27" s="88"/>
+      <c r="J27" s="88"/>
+      <c r="K27" s="88"/>
+      <c r="L27" s="88"/>
+      <c r="M27" s="88"/>
+      <c r="N27" s="88"/>
+      <c r="O27" s="88"/>
+      <c r="P27" s="89"/>
     </row>
     <row r="28" spans="1:17" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A28" s="69" t="s">
+      <c r="A28" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="70"/>
-      <c r="C28" s="70"/>
-      <c r="D28" s="70"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="70"/>
-      <c r="H28" s="70"/>
-      <c r="I28" s="70"/>
-      <c r="J28" s="70"/>
-      <c r="K28" s="70"/>
-      <c r="L28" s="70"/>
-      <c r="M28" s="70"/>
-      <c r="N28" s="70"/>
-      <c r="O28" s="70"/>
-      <c r="P28" s="71"/>
+      <c r="B28" s="73"/>
+      <c r="C28" s="73"/>
+      <c r="D28" s="73"/>
+      <c r="E28" s="73"/>
+      <c r="F28" s="73"/>
+      <c r="G28" s="73"/>
+      <c r="H28" s="73"/>
+      <c r="I28" s="73"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="73"/>
+      <c r="L28" s="73"/>
+      <c r="M28" s="73"/>
+      <c r="N28" s="73"/>
+      <c r="O28" s="73"/>
+      <c r="P28" s="74"/>
     </row>
     <row r="29" spans="1:17" ht="26.25" customHeight="1">
       <c r="A29" s="96" t="s">
         <v>64</v>
       </c>
       <c r="B29" s="97"/>
-      <c r="C29" s="100"/>
-      <c r="D29" s="100"/>
-      <c r="E29" s="100"/>
-      <c r="F29" s="100"/>
-      <c r="G29" s="100"/>
-      <c r="H29" s="100"/>
-      <c r="I29" s="100"/>
-      <c r="J29" s="102" t="s">
+      <c r="C29" s="104"/>
+      <c r="D29" s="104"/>
+      <c r="E29" s="104"/>
+      <c r="F29" s="104"/>
+      <c r="G29" s="104"/>
+      <c r="H29" s="104"/>
+      <c r="I29" s="105"/>
+      <c r="J29" s="100" t="s">
         <v>65</v>
       </c>
-      <c r="K29" s="103"/>
-      <c r="L29" s="103"/>
-      <c r="M29" s="106"/>
-      <c r="N29" s="106"/>
-      <c r="O29" s="106"/>
-      <c r="P29" s="107"/>
+      <c r="K29" s="101"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="108"/>
+      <c r="N29" s="108"/>
+      <c r="O29" s="108"/>
+      <c r="P29" s="109"/>
     </row>
     <row r="30" spans="1:17" ht="23.25" customHeight="1">
-      <c r="A30" s="98"/>
+      <c r="A30" s="98" t="s">
+        <v>67</v>
+      </c>
       <c r="B30" s="99"/>
-      <c r="C30" s="101"/>
-      <c r="D30" s="101"/>
-      <c r="E30" s="101"/>
-      <c r="F30" s="101"/>
-      <c r="G30" s="101"/>
-      <c r="H30" s="101"/>
-      <c r="I30" s="101"/>
-      <c r="J30" s="104"/>
-      <c r="K30" s="105"/>
-      <c r="L30" s="105"/>
-      <c r="M30" s="108"/>
-      <c r="N30" s="108"/>
-      <c r="O30" s="108"/>
-      <c r="P30" s="109"/>
-    </row>
-    <row r="31" spans="1:17" s="3" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A31" s="87" t="s">
+      <c r="C30" s="106"/>
+      <c r="D30" s="106"/>
+      <c r="E30" s="106"/>
+      <c r="F30" s="106"/>
+      <c r="G30" s="106"/>
+      <c r="H30" s="106"/>
+      <c r="I30" s="107"/>
+      <c r="J30" s="102" t="s">
+        <v>67</v>
+      </c>
+      <c r="K30" s="103"/>
+      <c r="L30" s="103"/>
+      <c r="M30" s="110"/>
+      <c r="N30" s="110"/>
+      <c r="O30" s="110"/>
+      <c r="P30" s="111"/>
+    </row>
+    <row r="31" spans="1:17" ht="7.2" customHeight="1">
+      <c r="A31" s="112"/>
+      <c r="B31" s="113"/>
+      <c r="C31" s="132"/>
+      <c r="D31" s="132"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="132"/>
+      <c r="G31" s="132"/>
+      <c r="H31" s="132"/>
+      <c r="I31" s="133"/>
+      <c r="J31" s="114"/>
+      <c r="K31" s="114"/>
+      <c r="L31" s="114"/>
+      <c r="M31" s="115"/>
+      <c r="N31" s="115"/>
+      <c r="O31" s="115"/>
+      <c r="P31" s="116"/>
+    </row>
+    <row r="32" spans="1:17" ht="37.799999999999997" customHeight="1">
+      <c r="A32" s="117" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" s="118"/>
+      <c r="C32" s="129"/>
+      <c r="D32" s="129"/>
+      <c r="E32" s="129"/>
+      <c r="F32" s="129"/>
+      <c r="G32" s="129"/>
+      <c r="H32" s="129"/>
+      <c r="I32" s="134"/>
+      <c r="J32" s="119" t="s">
+        <v>68</v>
+      </c>
+      <c r="K32" s="119"/>
+      <c r="L32" s="119"/>
+      <c r="M32" s="130"/>
+      <c r="N32" s="130"/>
+      <c r="O32" s="130"/>
+      <c r="P32" s="131"/>
+    </row>
+    <row r="33" spans="1:16" ht="32.4" customHeight="1">
+      <c r="A33" s="112"/>
+      <c r="B33" s="113"/>
+      <c r="C33" s="129"/>
+      <c r="D33" s="129"/>
+      <c r="E33" s="129"/>
+      <c r="F33" s="129"/>
+      <c r="G33" s="129"/>
+      <c r="H33" s="129"/>
+      <c r="I33" s="134"/>
+      <c r="J33" s="114"/>
+      <c r="K33" s="114"/>
+      <c r="L33" s="114"/>
+      <c r="M33" s="130"/>
+      <c r="N33" s="130"/>
+      <c r="O33" s="130"/>
+      <c r="P33" s="131"/>
+    </row>
+    <row r="34" spans="1:16" ht="6" customHeight="1" thickBot="1">
+      <c r="A34" s="123"/>
+      <c r="B34" s="124"/>
+      <c r="C34" s="125"/>
+      <c r="D34" s="125"/>
+      <c r="E34" s="125"/>
+      <c r="F34" s="125"/>
+      <c r="G34" s="125"/>
+      <c r="H34" s="125"/>
+      <c r="I34" s="135"/>
+      <c r="J34" s="126"/>
+      <c r="K34" s="126"/>
+      <c r="L34" s="126"/>
+      <c r="M34" s="127"/>
+      <c r="N34" s="127"/>
+      <c r="O34" s="127"/>
+      <c r="P34" s="128"/>
+    </row>
+    <row r="35" spans="1:16" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A35" s="120" t="s">
         <v>66</v>
       </c>
-      <c r="B31" s="88"/>
-      <c r="C31" s="88"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="88"/>
-      <c r="J31" s="88"/>
-      <c r="K31" s="88"/>
-      <c r="L31" s="88"/>
-      <c r="M31" s="88"/>
-      <c r="N31" s="88"/>
-      <c r="O31" s="88"/>
-      <c r="P31" s="89"/>
-    </row>
-    <row r="32" spans="1:17" ht="18.75" customHeight="1">
-      <c r="A32" s="90"/>
-      <c r="B32" s="91"/>
-      <c r="C32" s="91"/>
-      <c r="D32" s="91"/>
-      <c r="E32" s="91"/>
-      <c r="F32" s="91"/>
-      <c r="G32" s="91"/>
-      <c r="H32" s="91"/>
-      <c r="I32" s="91"/>
-      <c r="J32" s="91"/>
-      <c r="K32" s="91"/>
-      <c r="L32" s="91"/>
-      <c r="M32" s="91"/>
-      <c r="N32" s="91"/>
-      <c r="O32" s="91"/>
-      <c r="P32" s="92"/>
-    </row>
-    <row r="33" spans="1:16" ht="19.5" customHeight="1">
-      <c r="A33" s="90"/>
-      <c r="B33" s="91"/>
-      <c r="C33" s="91"/>
-      <c r="D33" s="91"/>
-      <c r="E33" s="91"/>
-      <c r="F33" s="91"/>
-      <c r="G33" s="91"/>
-      <c r="H33" s="91"/>
-      <c r="I33" s="91"/>
-      <c r="J33" s="91"/>
-      <c r="K33" s="91"/>
-      <c r="L33" s="91"/>
-      <c r="M33" s="91"/>
-      <c r="N33" s="91"/>
-      <c r="O33" s="91"/>
-      <c r="P33" s="92"/>
-    </row>
-    <row r="34" spans="1:16" ht="13.5" thickBot="1">
-      <c r="A34" s="93"/>
-      <c r="B34" s="94"/>
-      <c r="C34" s="94"/>
-      <c r="D34" s="94"/>
-      <c r="E34" s="94"/>
-      <c r="F34" s="94"/>
-      <c r="G34" s="94"/>
-      <c r="H34" s="94"/>
-      <c r="I34" s="94"/>
-      <c r="J34" s="94"/>
-      <c r="K34" s="94"/>
-      <c r="L34" s="94"/>
-      <c r="M34" s="94"/>
-      <c r="N34" s="94"/>
-      <c r="O34" s="94"/>
-      <c r="P34" s="95"/>
-    </row>
-    <row r="35" spans="1:16">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-    </row>
-    <row r="36" spans="1:16">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4"/>
-      <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
-    </row>
-    <row r="37" spans="1:16">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-    </row>
-    <row r="38" spans="1:16">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="4"/>
-      <c r="M38" s="4"/>
-      <c r="N38" s="4"/>
+      <c r="B35" s="121"/>
+      <c r="C35" s="121"/>
+      <c r="D35" s="121"/>
+      <c r="E35" s="121"/>
+      <c r="F35" s="121"/>
+      <c r="G35" s="121"/>
+      <c r="H35" s="121"/>
+      <c r="I35" s="121"/>
+      <c r="J35" s="121"/>
+      <c r="K35" s="121"/>
+      <c r="L35" s="121"/>
+      <c r="M35" s="121"/>
+      <c r="N35" s="121"/>
+      <c r="O35" s="121"/>
+      <c r="P35" s="122"/>
+    </row>
+    <row r="36" spans="1:16" ht="18.75" customHeight="1">
+      <c r="A36" s="90"/>
+      <c r="B36" s="91"/>
+      <c r="C36" s="91"/>
+      <c r="D36" s="91"/>
+      <c r="E36" s="91"/>
+      <c r="F36" s="91"/>
+      <c r="G36" s="91"/>
+      <c r="H36" s="91"/>
+      <c r="I36" s="91"/>
+      <c r="J36" s="91"/>
+      <c r="K36" s="91"/>
+      <c r="L36" s="91"/>
+      <c r="M36" s="91"/>
+      <c r="N36" s="91"/>
+      <c r="O36" s="91"/>
+      <c r="P36" s="92"/>
+    </row>
+    <row r="37" spans="1:16" ht="19.5" customHeight="1">
+      <c r="A37" s="90"/>
+      <c r="B37" s="91"/>
+      <c r="C37" s="91"/>
+      <c r="D37" s="91"/>
+      <c r="E37" s="91"/>
+      <c r="F37" s="91"/>
+      <c r="G37" s="91"/>
+      <c r="H37" s="91"/>
+      <c r="I37" s="91"/>
+      <c r="J37" s="91"/>
+      <c r="K37" s="91"/>
+      <c r="L37" s="91"/>
+      <c r="M37" s="91"/>
+      <c r="N37" s="91"/>
+      <c r="O37" s="91"/>
+      <c r="P37" s="92"/>
+    </row>
+    <row r="38" spans="1:16" ht="13.8" thickBot="1">
+      <c r="A38" s="93"/>
+      <c r="B38" s="94"/>
+      <c r="C38" s="94"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="94"/>
+      <c r="F38" s="94"/>
+      <c r="G38" s="94"/>
+      <c r="H38" s="94"/>
+      <c r="I38" s="94"/>
+      <c r="J38" s="94"/>
+      <c r="K38" s="94"/>
+      <c r="L38" s="94"/>
+      <c r="M38" s="94"/>
+      <c r="N38" s="94"/>
+      <c r="O38" s="94"/>
+      <c r="P38" s="95"/>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" s="4"/>
@@ -3748,15 +3878,87 @@
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
       <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+    </row>
+    <row r="49" spans="1:14">
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+    </row>
+    <row r="50" spans="1:14">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="54">
-    <mergeCell ref="A31:P31"/>
-    <mergeCell ref="A32:P34"/>
-    <mergeCell ref="A29:B30"/>
-    <mergeCell ref="C29:I30"/>
-    <mergeCell ref="J29:L30"/>
-    <mergeCell ref="M29:P30"/>
+  <mergeCells count="62">
+    <mergeCell ref="A35:P35"/>
+    <mergeCell ref="A36:P38"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C30:I30"/>
+    <mergeCell ref="M29:P29"/>
+    <mergeCell ref="M30:P30"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="J32:L32"/>
+    <mergeCell ref="C32:I33"/>
+    <mergeCell ref="M32:P33"/>
     <mergeCell ref="G18:I18"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A19:C19"/>

</xml_diff>